<commit_message>
V3 foundation: real purchase costs, demo data removed, per-user chat schema
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018W7NxFXoeXGaFsJkP1KqtT
</commit_message>
<xml_diff>
--- a/data/Data_base_products.xlsx
+++ b/data/Data_base_products.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabien\Desktop\Kaviari Cellar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B97A3F52-AE1F-4B43-BF73-DBFA44C3D5CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20786B4-ED57-4BF4-B062-08867F8B0795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="description" sheetId="1" r:id="rId1"/>
+    <sheet name="Cost" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$3:$E$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cost!$A$3:$H$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">description!$A$3:$E$88</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="109">
   <si>
     <t>PR Code</t>
   </si>
@@ -360,12 +362,24 @@
   </si>
   <si>
     <t>Packing / box</t>
+  </si>
+  <si>
+    <t>Cost / kg</t>
+  </si>
+  <si>
+    <t>Weight / Tin</t>
+  </si>
+  <si>
+    <t>Cost / Tin</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="_-[$€-2]\ * #,##0.00_-;\-[$€-2]\ * #,##0.00_-;_-[$€-2]\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -431,7 +445,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -441,6 +455,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -775,7 +790,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A3:G88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -969,7 +983,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9416</v>
       </c>
@@ -983,6 +997,8 @@
       <c r="E11" s="3" t="s">
         <v>88</v>
       </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
@@ -1007,7 +1023,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>8579</v>
       </c>
@@ -1021,8 +1037,10 @@
       <c r="E13" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>9295</v>
       </c>
@@ -1036,6 +1054,8 @@
       <c r="E14" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
@@ -1083,7 +1103,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>8576</v>
       </c>
@@ -1097,8 +1117,10 @@
       <c r="E17" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>8580</v>
       </c>
@@ -1112,8 +1134,10 @@
       <c r="E18" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>9396</v>
       </c>
@@ -1127,8 +1151,10 @@
       <c r="E19" s="3" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>8577</v>
       </c>
@@ -1142,6 +1168,8 @@
       <c r="E20" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
@@ -1166,7 +1194,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>8574</v>
       </c>
@@ -1180,8 +1208,10 @@
       <c r="E22" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>8575</v>
       </c>
@@ -1195,8 +1225,10 @@
       <c r="E23" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>8581</v>
       </c>
@@ -1210,8 +1242,10 @@
       <c r="E24" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>8919</v>
       </c>
@@ -1225,8 +1259,10 @@
       <c r="E25" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>8920</v>
       </c>
@@ -1240,6 +1276,8 @@
       <c r="E26" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
@@ -1264,7 +1302,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>9201</v>
       </c>
@@ -1278,8 +1316,10 @@
       <c r="E28" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>9202</v>
       </c>
@@ -1293,6 +1333,8 @@
       <c r="E29" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
@@ -1455,7 +1497,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>3168</v>
       </c>
@@ -1469,6 +1511,8 @@
       <c r="E37" s="3" t="s">
         <v>95</v>
       </c>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
@@ -1516,7 +1560,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>3202</v>
       </c>
@@ -1530,8 +1574,10 @@
       <c r="E40" s="3" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>3208</v>
       </c>
@@ -1545,6 +1591,8 @@
       <c r="E41" s="3" t="s">
         <v>95</v>
       </c>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
@@ -1569,7 +1617,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>3254</v>
       </c>
@@ -1583,6 +1631,8 @@
       <c r="E43" s="3" t="s">
         <v>95</v>
       </c>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
@@ -1607,7 +1657,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>3916</v>
       </c>
@@ -1621,8 +1671,10 @@
       <c r="E45" s="3" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>4062</v>
       </c>
@@ -1636,6 +1688,8 @@
       <c r="E46" s="3" t="s">
         <v>103</v>
       </c>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
@@ -1752,7 +1806,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>5917</v>
       </c>
@@ -1766,8 +1820,10 @@
       <c r="E52" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>5918</v>
       </c>
@@ -1781,8 +1837,10 @@
       <c r="E53" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>5919</v>
       </c>
@@ -1796,8 +1854,10 @@
       <c r="E54" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>6181</v>
       </c>
@@ -1811,8 +1871,10 @@
       <c r="E55" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>6345</v>
       </c>
@@ -1826,8 +1888,10 @@
       <c r="E56" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
         <v>6346</v>
       </c>
@@ -1841,6 +1905,8 @@
       <c r="E57" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
@@ -1888,7 +1954,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
         <v>6914</v>
       </c>
@@ -1902,6 +1968,8 @@
       <c r="E60" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1">
@@ -1949,7 +2017,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>7580</v>
       </c>
@@ -1963,8 +2031,10 @@
       <c r="E63" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="1">
         <v>7581</v>
       </c>
@@ -1978,8 +2048,10 @@
       <c r="E64" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>7592</v>
       </c>
@@ -1993,8 +2065,10 @@
       <c r="E65" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
         <v>7605</v>
       </c>
@@ -2008,6 +2082,8 @@
       <c r="E66" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1">
@@ -2032,7 +2108,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>7764</v>
       </c>
@@ -2046,8 +2122,10 @@
       <c r="E68" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>7767</v>
       </c>
@@ -2061,8 +2139,10 @@
       <c r="E69" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
         <v>7883</v>
       </c>
@@ -2076,6 +2156,8 @@
       <c r="E70" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
@@ -2100,7 +2182,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>8384</v>
       </c>
@@ -2114,6 +2196,8 @@
       <c r="E72" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
@@ -2184,7 +2268,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
         <v>8756</v>
       </c>
@@ -2198,6 +2282,8 @@
       <c r="E76" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
@@ -2245,7 +2331,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
         <v>9088</v>
       </c>
@@ -2259,8 +2345,10 @@
       <c r="E79" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>9089</v>
       </c>
@@ -2274,8 +2362,10 @@
       <c r="E80" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
         <v>9101</v>
       </c>
@@ -2289,8 +2379,10 @@
       <c r="E81" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
         <v>9296</v>
       </c>
@@ -2304,8 +2396,10 @@
       <c r="E82" s="3" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1">
         <v>9428</v>
       </c>
@@ -2319,6 +2413,8 @@
       <c r="E83" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="1">
@@ -2389,7 +2485,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>9017</v>
       </c>
@@ -2403,6 +2499,8 @@
       <c r="E87" s="3" t="s">
         <v>94</v>
       </c>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
@@ -2428,13 +2526,1967 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:E88" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Caviar"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A3:E88" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}">
+  <dimension ref="A3:H88"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="68.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="15.140625" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3193</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="5">
+        <v>765</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H4" s="5">
+        <f>G4*F4</f>
+        <v>95.625</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>3134</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F5" s="5">
+        <v>830</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H5" s="5">
+        <f>G5*F5</f>
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>3126</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="5">
+        <v>830</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H6" s="5">
+        <f t="shared" ref="H6:H7" si="0">G6*F6</f>
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>3343</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F7" s="5">
+        <v>830</v>
+      </c>
+      <c r="G7" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="H7" s="5">
+        <f t="shared" si="0"/>
+        <v>16.600000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>1216</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="5">
+        <v>765</v>
+      </c>
+      <c r="G8" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H8" s="5">
+        <f>G8*F8</f>
+        <v>22.95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>7715</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G9" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H9" s="5">
+        <f>G9*F9</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>3127</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" s="5">
+        <v>830</v>
+      </c>
+      <c r="G10" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H10" s="5">
+        <f>G10*F10</f>
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>9416</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>3148</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F12" s="5">
+        <v>525</v>
+      </c>
+      <c r="G12" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H12" s="5">
+        <f>G12*F12</f>
+        <v>15.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>8579</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F13" s="5"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>9295</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>9011</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F15" s="5">
+        <v>830</v>
+      </c>
+      <c r="G15" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H15" s="5">
+        <f>G15*F15</f>
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>3133</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F16" s="5">
+        <v>765</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H16" s="5">
+        <f>G16*F16</f>
+        <v>38.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>8576</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="5"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>8580</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F18" s="5"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="5"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>9396</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>8577</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>7881</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F21" s="5">
+        <v>2900</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H21" s="5">
+        <f>G21*F21</f>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>8574</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="5"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>8575</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" s="5"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>8581</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="5"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>8919</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>8920</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26" s="5"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="5"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>3220</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F27" s="5">
+        <v>2900</v>
+      </c>
+      <c r="G27" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H27" s="5">
+        <f>G27*F27</f>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>9201</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F28" s="5"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="5"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>9202</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" s="5"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>3342</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F30" s="5">
+        <v>865</v>
+      </c>
+      <c r="G30" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="H30" s="5">
+        <f>G30*F30</f>
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>1215</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" s="5">
+        <v>525</v>
+      </c>
+      <c r="G31" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H31" s="5">
+        <f>G31*F31</f>
+        <v>15.75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>3119</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F32" s="5">
+        <v>986.67</v>
+      </c>
+      <c r="G32" s="3">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H32" s="5">
+        <f t="shared" ref="H32:H33" si="1">G32*F32</f>
+        <v>14.800049999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>3120</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F33" s="5">
+        <v>830</v>
+      </c>
+      <c r="G33" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H33" s="5">
+        <f t="shared" si="1"/>
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>3123</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F34" s="5">
+        <v>765</v>
+      </c>
+      <c r="G34" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="H34" s="5">
+        <f>G34*F34</f>
+        <v>76.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>3124</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F35" s="5">
+        <v>830</v>
+      </c>
+      <c r="G35" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="H35" s="5">
+        <f>G35*F35</f>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>3135</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F36" s="5">
+        <v>525</v>
+      </c>
+      <c r="G36" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H36" s="5">
+        <f>G36*F36</f>
+        <v>26.25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>3168</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F37" s="5"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="5"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>3169</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F38" s="5">
+        <v>830</v>
+      </c>
+      <c r="G38" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H38" s="5">
+        <f>G38*F38</f>
+        <v>207.5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>3192</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E39" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F39" s="5">
+        <v>765</v>
+      </c>
+      <c r="G39" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H39" s="5">
+        <f>G39*F39</f>
+        <v>191.25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>3202</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F40" s="5"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="5"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>3208</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E41" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F41" s="5"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="5"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>3227</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F42" s="5">
+        <v>2900</v>
+      </c>
+      <c r="G42" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H42" s="5">
+        <f>G42*F42</f>
+        <v>362.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>3254</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F43" s="5"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="5"/>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>3274</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F44" s="5">
+        <v>2900</v>
+      </c>
+      <c r="G44" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H44" s="5">
+        <f>G44*F44</f>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>3916</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F45" s="5"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="5"/>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>4062</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F46" s="5"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="5"/>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>4160</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F47" s="5">
+        <v>765</v>
+      </c>
+      <c r="G47" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H47" s="5">
+        <f>G47*F47</f>
+        <v>382.5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>4291</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F48" s="5">
+        <v>525</v>
+      </c>
+      <c r="G48" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H48" s="5">
+        <f>G48*F48</f>
+        <v>262.5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>4298</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F49" s="5">
+        <v>830</v>
+      </c>
+      <c r="G49" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H49" s="5">
+        <f>G49*F49</f>
+        <v>415</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>4403</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E50" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F50" s="5">
+        <v>680</v>
+      </c>
+      <c r="G50" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H50" s="5">
+        <f>G50*F50</f>
+        <v>20.399999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>4404</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F51" s="5">
+        <v>680</v>
+      </c>
+      <c r="G51" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H51" s="5">
+        <f>G51*F51</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>5917</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F52" s="5"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="5"/>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>5918</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F53" s="5"/>
+      <c r="G53" s="3"/>
+      <c r="H53" s="5"/>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>5919</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F54" s="5"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="5"/>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>6181</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F55" s="5"/>
+      <c r="G55" s="3"/>
+      <c r="H55" s="5"/>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>6345</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E56" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F56" s="5"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="5"/>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>6346</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E57" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F57" s="5"/>
+      <c r="G57" s="3"/>
+      <c r="H57" s="5"/>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>6863</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E58" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F58" s="5">
+        <v>830</v>
+      </c>
+      <c r="G58" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H58" s="5">
+        <f t="shared" ref="H58:H59" si="2">G58*F58</f>
+        <v>207.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>6913</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F59" s="5">
+        <v>830</v>
+      </c>
+      <c r="G59" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="H59" s="5">
+        <f t="shared" si="2"/>
+        <v>8.3000000000000007</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>6914</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E60" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F60" s="5"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="5"/>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>6988</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E61" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F61" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G61" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H61" s="5">
+        <f t="shared" ref="H61:H62" si="3">G61*F61</f>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>6989</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F62" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G62" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H62" s="5">
+        <f t="shared" si="3"/>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>7580</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E63" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F63" s="5"/>
+      <c r="G63" s="3"/>
+      <c r="H63" s="5"/>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>7581</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E64" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F64" s="5"/>
+      <c r="G64" s="3"/>
+      <c r="H64" s="5"/>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>7592</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E65" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F65" s="5"/>
+      <c r="G65" s="3"/>
+      <c r="H65" s="5"/>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>7605</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C66" s="2"/>
+      <c r="D66" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F66" s="5"/>
+      <c r="G66" s="3"/>
+      <c r="H66" s="5"/>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>7714</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E67" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F67" s="5">
+        <v>830</v>
+      </c>
+      <c r="G67" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H67" s="5">
+        <f>G67*F67</f>
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>7764</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F68" s="5"/>
+      <c r="G68" s="3"/>
+      <c r="H68" s="5"/>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>7767</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F69" s="5"/>
+      <c r="G69" s="3"/>
+      <c r="H69" s="5"/>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>7883</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C70" s="2"/>
+      <c r="D70" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F70" s="5"/>
+      <c r="G70" s="3"/>
+      <c r="H70" s="5"/>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>8173</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F71" s="5">
+        <v>986.67</v>
+      </c>
+      <c r="G71" s="3">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H71" s="5">
+        <f>G71*F71</f>
+        <v>14.800049999999999</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>8384</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C72" s="2"/>
+      <c r="D72" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F72" s="5"/>
+      <c r="G72" s="3"/>
+      <c r="H72" s="5"/>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>8510</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F73" s="5">
+        <v>1200</v>
+      </c>
+      <c r="G73" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H73" s="5">
+        <f>G73*F73</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>8559</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F74" s="5">
+        <v>525</v>
+      </c>
+      <c r="G74" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H74" s="5">
+        <f t="shared" ref="H74:H75" si="4">G74*F74</f>
+        <v>26.25</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>8669</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C75" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F75" s="5">
+        <v>525</v>
+      </c>
+      <c r="G75" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H75" s="5">
+        <f t="shared" si="4"/>
+        <v>15.75</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>8756</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C76" s="2"/>
+      <c r="D76" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F76" s="5"/>
+      <c r="G76" s="3"/>
+      <c r="H76" s="5"/>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>8992</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E77" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F77" s="5">
+        <v>525</v>
+      </c>
+      <c r="G77" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="H77" s="5">
+        <f>G77*F77</f>
+        <v>26.25</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>8993</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F78" s="5">
+        <v>830</v>
+      </c>
+      <c r="G78" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="H78" s="5">
+        <f>G78*F78</f>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>9088</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C79" s="2"/>
+      <c r="D79" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E79" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F79" s="5"/>
+      <c r="G79" s="3"/>
+      <c r="H79" s="5"/>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>9089</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E80" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F80" s="5"/>
+      <c r="G80" s="3"/>
+      <c r="H80" s="5"/>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>9101</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C81" s="2"/>
+      <c r="D81" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F81" s="5"/>
+      <c r="G81" s="3"/>
+      <c r="H81" s="5"/>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>9296</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E82" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F82" s="5"/>
+      <c r="G82" s="3"/>
+      <c r="H82" s="5"/>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>9428</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F83" s="5"/>
+      <c r="G83" s="3"/>
+      <c r="H83" s="5"/>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>4186</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D84" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F84" s="5">
+        <v>986.67</v>
+      </c>
+      <c r="G84" s="3">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="H84" s="5">
+        <f>G84*F84</f>
+        <v>14.800049999999999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>7712</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F85" s="5">
+        <v>765</v>
+      </c>
+      <c r="G85" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H85" s="5">
+        <f>G85*F85</f>
+        <v>22.95</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>7713</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D86" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F86" s="5">
+        <v>830</v>
+      </c>
+      <c r="G86" s="3">
+        <v>0.03</v>
+      </c>
+      <c r="H86" s="5">
+        <f>G86*F86</f>
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>9017</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F87" s="5"/>
+      <c r="G87" s="3"/>
+      <c r="H87" s="5"/>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>3344</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C88" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D88" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F88" s="5">
+        <v>625</v>
+      </c>
+      <c r="G88" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="H88" s="5">
+        <f>G88*F88</f>
+        <v>12.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:H88" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sync catalog from updated product workbook; Code column in every table
Maintenance v7 upserts products by PR code from the refreshed
Data_base_products.xlsx (7 new: unpasteurized Kristal 30/50 g and the
Baenki 125 g - 1.8 kg range; sizes filled for empty-tin marketing
items) without touching movements, lots, forecasts or accounts. A Code
column now leads the planner table, PO detail lines, receive dialog and
all import previews (stock take, sales, price changes).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018W7NxFXoeXGaFsJkP1KqtT
</commit_message>
<xml_diff>
--- a/data/Data_base_products.xlsx
+++ b/data/Data_base_products.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabien\Desktop\Kaviari Cellar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B20786B4-ED57-4BF4-B062-08867F8B0795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1642F5D7-4582-4822-97FB-130A530D86DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1C395D8-19D5-4EE8-9504-7413A88F6FBD}"/>
   </bookViews>
   <sheets>
     <sheet name="description" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Cost!$A$3:$H$88</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">description!$A$3:$E$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">description!$A$3:$E$95</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="654" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="116">
   <si>
     <t>PR Code</t>
   </si>
@@ -371,6 +371,27 @@
   </si>
   <si>
     <t>Cost / Tin</t>
+  </si>
+  <si>
+    <t>Kaviari Kristal caviar 50 g/tin (unpasteurized)</t>
+  </si>
+  <si>
+    <t>Kaviari Caviar Kristal (30 g/tin)[unpasteurized]</t>
+  </si>
+  <si>
+    <t>Kaviari Baenki Caviar 1.8 KG/Tin</t>
+  </si>
+  <si>
+    <t>Kaviari Baenki caviar 1 KG/Tin</t>
+  </si>
+  <si>
+    <t>Kaviari Baenki caviar 500 g/Tin</t>
+  </si>
+  <si>
+    <t>Kaviari Baenki 250 g/Tin</t>
+  </si>
+  <si>
+    <t>Kaviari Baenki caviar 125 g/Tin</t>
   </si>
 </sst>
 </file>
@@ -418,7 +439,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -441,11 +462,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -456,6 +490,17 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -790,7 +835,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}">
-  <dimension ref="A3:G88"/>
+  <dimension ref="A3:G95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="68.140625" bestFit="1" customWidth="1"/>
@@ -2309,25 +2354,25 @@
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
+      <c r="A78" s="8">
         <v>8993</v>
       </c>
-      <c r="B78" s="2" t="s">
+      <c r="B78" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E78" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F78" s="3">
+      <c r="D78" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E78" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="F78" s="10">
         <v>12</v>
       </c>
-      <c r="G78" s="3" t="s">
+      <c r="G78" s="10" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2525,15 +2570,176 @@
         <v>88</v>
       </c>
     </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" s="6">
+        <v>9573</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F89" s="3">
+        <v>24</v>
+      </c>
+      <c r="G89" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="6">
+        <v>3341</v>
+      </c>
+      <c r="B90" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F90" s="3">
+        <v>24</v>
+      </c>
+      <c r="G90" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>9582</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F91" s="11">
+        <v>1</v>
+      </c>
+      <c r="G91" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>9583</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F92" s="11">
+        <v>1</v>
+      </c>
+      <c r="G92" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>9584</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F93" s="11">
+        <v>2</v>
+      </c>
+      <c r="G93" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>9585</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F94" s="11">
+        <v>5</v>
+      </c>
+      <c r="G94" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>9586</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F95" s="11">
+        <v>12</v>
+      </c>
+      <c r="G95" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:E88" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}"/>
+  <autoFilter ref="A3:E95" xr:uid="{70808981-2AFB-4C59-8FC0-68C9336C3778}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}">
-  <dimension ref="A3:H88"/>
+  <dimension ref="A3:H95"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="68.140625" bestFit="1" customWidth="1"/>
@@ -4485,6 +4691,195 @@
         <v>12.5</v>
       </c>
     </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>9582</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C89" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D89" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E89" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F89" s="5">
+        <v>525</v>
+      </c>
+      <c r="G89" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="H89" s="12">
+        <f>G89*F89</f>
+        <v>945</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>9583</v>
+      </c>
+      <c r="B90" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D90" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F90" s="5">
+        <v>525</v>
+      </c>
+      <c r="G90" s="3">
+        <v>1</v>
+      </c>
+      <c r="H90" s="12">
+        <f t="shared" ref="H90:H95" si="5">G90*F90</f>
+        <v>525</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>9584</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C91" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D91" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F91" s="5">
+        <v>525</v>
+      </c>
+      <c r="G91" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H91" s="12">
+        <f t="shared" si="5"/>
+        <v>262.5</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>9585</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C92" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D92" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F92" s="5">
+        <v>525</v>
+      </c>
+      <c r="G92" s="3">
+        <v>0.25</v>
+      </c>
+      <c r="H92" s="12">
+        <f t="shared" si="5"/>
+        <v>131.25</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>9586</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C93" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D93" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F93" s="5">
+        <v>525</v>
+      </c>
+      <c r="G93" s="3">
+        <v>0.125</v>
+      </c>
+      <c r="H93" s="12">
+        <f t="shared" si="5"/>
+        <v>65.625</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="6">
+        <v>9573</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="C94" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D94" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E94" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F94" s="12">
+        <v>785</v>
+      </c>
+      <c r="G94" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="H94" s="12">
+        <f t="shared" si="5"/>
+        <v>39.25</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="6">
+        <v>3341</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E95" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="F95" s="12">
+        <v>785</v>
+      </c>
+      <c r="G95" s="11">
+        <v>0.03</v>
+      </c>
+      <c r="H95" s="12">
+        <f t="shared" si="5"/>
+        <v>23.55</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A3:H88" xr:uid="{5D728A83-21A1-4AAF-B2FC-CCC59733812F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>